<commit_message>
Updated skills for easier use. Loaded updated doc from google
</commit_message>
<xml_diff>
--- a/interviewees.xlsx
+++ b/interviewees.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4917448F-8626-4DCC-9B50-0637686830ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-78" yWindow="0" windowWidth="11676" windowHeight="13758" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-240" yWindow="-240" windowWidth="52080" windowHeight="21360" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Table for thesis" sheetId="1" r:id="rId1"/>
@@ -554,9 +554,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:J19"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.6"/>
+  <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.6"/>
   <sheetData>
-    <row r="1" spans="1:10" ht="15.6" x14ac:dyDescent="0.6">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.6">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -570,7 +570,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="15.6" x14ac:dyDescent="0.6">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.6">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -602,7 +602,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:10" ht="15.6" x14ac:dyDescent="0.6">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.6">
       <c r="A3" t="s">
         <v>14</v>
       </c>
@@ -616,7 +616,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="4" spans="1:10" ht="15.6" x14ac:dyDescent="0.6">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.6">
       <c r="A4" t="s">
         <v>16</v>
       </c>
@@ -630,7 +630,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="5" spans="1:10" ht="15.6" x14ac:dyDescent="0.6">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.6">
       <c r="A5" t="s">
         <v>17</v>
       </c>
@@ -650,7 +650,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="6" spans="1:10" ht="15.6" x14ac:dyDescent="0.6">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.6">
       <c r="A6" t="s">
         <v>18</v>
       </c>
@@ -664,7 +664,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="7" spans="1:10" ht="15.6" x14ac:dyDescent="0.6">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.6">
       <c r="A7" t="s">
         <v>19</v>
       </c>
@@ -678,7 +678,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="8" spans="1:10" ht="15.6" x14ac:dyDescent="0.6">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.6">
       <c r="A8" t="s">
         <v>20</v>
       </c>
@@ -692,7 +692,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="9" spans="1:10" ht="15.6" x14ac:dyDescent="0.6">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.6">
       <c r="A9" t="s">
         <v>21</v>
       </c>
@@ -703,7 +703,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="10" spans="1:10" ht="15.6" x14ac:dyDescent="0.6">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.6">
       <c r="A10" t="s">
         <v>22</v>
       </c>
@@ -717,7 +717,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="11" spans="1:10" ht="15.6" x14ac:dyDescent="0.6">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.6">
       <c r="A11" t="s">
         <v>23</v>
       </c>
@@ -731,7 +731,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="12" spans="1:10" ht="15.6" x14ac:dyDescent="0.6">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.6">
       <c r="A12" t="s">
         <v>24</v>
       </c>
@@ -745,7 +745,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="13" spans="1:10" ht="15.6" x14ac:dyDescent="0.6">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.6">
       <c r="A13" t="s">
         <v>25</v>
       </c>
@@ -759,7 +759,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="14" spans="1:10" ht="15.6" x14ac:dyDescent="0.6">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.6">
       <c r="A14" t="s">
         <v>26</v>
       </c>
@@ -773,7 +773,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="15" spans="1:10" ht="15.6" x14ac:dyDescent="0.6">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.6">
       <c r="A15" t="s">
         <v>27</v>
       </c>
@@ -790,7 +790,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="16" spans="1:10" ht="15.6" x14ac:dyDescent="0.6">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.6">
       <c r="A16" t="s">
         <v>28</v>
       </c>
@@ -804,7 +804,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="17" spans="1:9" ht="15.6" x14ac:dyDescent="0.6">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.6">
       <c r="A17" t="s">
         <v>29</v>
       </c>
@@ -818,7 +818,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="18" spans="1:9" ht="15.6" x14ac:dyDescent="0.6">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.6">
       <c r="A18" t="s">
         <v>30</v>
       </c>
@@ -838,7 +838,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="19" spans="1:9" ht="15.6" x14ac:dyDescent="0.6">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.6">
       <c r="A19" t="s">
         <v>31</v>
       </c>
@@ -863,9 +863,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:C18"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.6"/>
+  <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.6"/>
   <sheetData>
-    <row r="1" spans="1:3" ht="15.6" x14ac:dyDescent="0.6">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.6">
       <c r="A1" t="s">
         <v>32</v>
       </c>
@@ -876,7 +876,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="15.6" x14ac:dyDescent="0.6">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.6">
       <c r="A2" t="s">
         <v>14</v>
       </c>
@@ -887,7 +887,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="15.6" x14ac:dyDescent="0.6">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.6">
       <c r="A3" t="s">
         <v>16</v>
       </c>
@@ -895,7 +895,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="15.6" x14ac:dyDescent="0.6">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.6">
       <c r="A4" t="s">
         <v>17</v>
       </c>
@@ -906,7 +906,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="15.6" x14ac:dyDescent="0.6">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.6">
       <c r="A5" t="s">
         <v>18</v>
       </c>
@@ -917,7 +917,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="15.6" x14ac:dyDescent="0.6">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.6">
       <c r="A6" t="s">
         <v>19</v>
       </c>
@@ -928,7 +928,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="15.6" x14ac:dyDescent="0.6">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.6">
       <c r="A7" t="s">
         <v>20</v>
       </c>
@@ -939,7 +939,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="15.6" x14ac:dyDescent="0.6">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.6">
       <c r="A8" t="s">
         <v>21</v>
       </c>
@@ -950,7 +950,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="15.6" x14ac:dyDescent="0.6">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.6">
       <c r="A9" t="s">
         <v>22</v>
       </c>
@@ -961,7 +961,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="15.6" x14ac:dyDescent="0.6">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.6">
       <c r="A10" t="s">
         <v>23</v>
       </c>
@@ -972,7 +972,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="15.6" x14ac:dyDescent="0.6">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.6">
       <c r="A11" t="s">
         <v>24</v>
       </c>
@@ -983,7 +983,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="12" spans="1:3" ht="15.6" x14ac:dyDescent="0.6">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.6">
       <c r="A12" t="s">
         <v>25</v>
       </c>
@@ -994,7 +994,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="15.6" x14ac:dyDescent="0.6">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.6">
       <c r="A13" t="s">
         <v>26</v>
       </c>
@@ -1005,7 +1005,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="15.6" x14ac:dyDescent="0.6">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.6">
       <c r="A14" t="s">
         <v>27</v>
       </c>
@@ -1016,7 +1016,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="15.6" x14ac:dyDescent="0.6">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.6">
       <c r="A15" t="s">
         <v>28</v>
       </c>
@@ -1027,7 +1027,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="15.6" x14ac:dyDescent="0.6">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.6">
       <c r="A16" t="s">
         <v>29</v>
       </c>
@@ -1038,7 +1038,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="17" spans="1:3" ht="15.6" x14ac:dyDescent="0.6">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.6">
       <c r="A17" t="s">
         <v>30</v>
       </c>
@@ -1049,7 +1049,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="18" spans="1:3" ht="15.6" x14ac:dyDescent="0.6">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.6">
       <c r="A18" t="s">
         <v>31</v>
       </c>

</xml_diff>

<commit_message>
added auxiliary resources again
</commit_message>
<xml_diff>
--- a/interviewees.xlsx
+++ b/interviewees.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4917448F-8626-4DCC-9B50-0637686830ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-240" yWindow="-240" windowWidth="52080" windowHeight="21360" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="26010" windowHeight="20985" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Table for thesis" sheetId="1" r:id="rId1"/>
@@ -554,9 +554,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:J19"/>
-  <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.6"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.6">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -570,7 +570,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.6">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -602,7 +602,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.6">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>14</v>
       </c>
@@ -616,7 +616,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.6">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>16</v>
       </c>
@@ -630,7 +630,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.6">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>17</v>
       </c>
@@ -650,7 +650,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.6">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>18</v>
       </c>
@@ -664,7 +664,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.6">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>19</v>
       </c>
@@ -678,7 +678,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.6">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>20</v>
       </c>
@@ -692,7 +692,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.6">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>21</v>
       </c>
@@ -703,7 +703,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.6">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>22</v>
       </c>
@@ -717,7 +717,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.6">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>23</v>
       </c>
@@ -731,7 +731,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.6">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>24</v>
       </c>
@@ -745,7 +745,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.6">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>25</v>
       </c>
@@ -759,7 +759,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.6">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>26</v>
       </c>
@@ -773,7 +773,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.6">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>27</v>
       </c>
@@ -790,7 +790,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.6">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>28</v>
       </c>
@@ -804,7 +804,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.6">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>29</v>
       </c>
@@ -818,7 +818,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.6">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>30</v>
       </c>
@@ -838,7 +838,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.6">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>31</v>
       </c>
@@ -863,9 +863,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:C18"/>
-  <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.6"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.6">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>32</v>
       </c>
@@ -876,7 +876,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.6">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>14</v>
       </c>
@@ -887,7 +887,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.6">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>16</v>
       </c>
@@ -895,7 +895,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.6">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>17</v>
       </c>
@@ -906,7 +906,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.6">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>18</v>
       </c>
@@ -917,7 +917,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.6">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>19</v>
       </c>
@@ -928,7 +928,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.6">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>20</v>
       </c>
@@ -939,7 +939,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.6">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>21</v>
       </c>
@@ -950,7 +950,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.6">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>22</v>
       </c>
@@ -961,7 +961,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.6">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>23</v>
       </c>
@@ -972,7 +972,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.6">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>24</v>
       </c>
@@ -983,7 +983,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.6">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>25</v>
       </c>
@@ -994,7 +994,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.6">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>26</v>
       </c>
@@ -1005,7 +1005,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.6">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>27</v>
       </c>
@@ -1016,7 +1016,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.6">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>28</v>
       </c>
@@ -1027,7 +1027,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.6">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>29</v>
       </c>
@@ -1038,7 +1038,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.6">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>30</v>
       </c>
@@ -1049,7 +1049,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.6">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>31</v>
       </c>

</xml_diff>